<commit_message>
20260922_추석전 pipeline 수정 정지_bigquery 날짜 범위 확장.
</commit_message>
<xml_diff>
--- a/30_output_share/06_BRONZE노출감사.xlsx
+++ b/30_output_share/06_BRONZE노출감사.xlsx
@@ -541,7 +541,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BRONZE 노출감사 — 전 원천 1254컬럼 (2026-09-21)</t>
+          <t>BRONZE 노출감사 — 전 원천 1254컬럼 (2026-09-22)</t>
         </is>
       </c>
     </row>
@@ -658,11 +658,11 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>542</v>
+        <v>492</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>43.2%</t>
+          <t>39.2%</t>
         </is>
       </c>
     </row>
@@ -703,11 +703,11 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>8.0%</t>
         </is>
       </c>
     </row>
@@ -849,7 +849,7 @@
         <v>6</v>
       </c>
       <c r="G20" t="n">
-        <v>522</v>
+        <v>472</v>
       </c>
       <c r="H20" t="n">
         <v>58</v>
@@ -858,7 +858,7 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="K20" t="n">
         <v>1064</v>
@@ -11265,19 +11265,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D79" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D79" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E79" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F79" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -11713,19 +11713,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D93" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D93" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E93" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F93" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -12001,19 +12001,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D102" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D102" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E102" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F102" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -13761,19 +13761,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D157" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D157" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E157" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F157" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -14177,19 +14177,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D170" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D170" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E170" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F170" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -14753,19 +14753,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D188" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D188" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E188" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F188" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -15297,19 +15297,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D205" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D205" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E205" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F205" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -15777,19 +15777,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D220" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D220" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E220" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F220" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -16481,19 +16481,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D242" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D242" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E242" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F242" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -17345,19 +17345,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D269" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D269" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E269" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F269" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -17761,19 +17761,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D282" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D282" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E282" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F282" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -18337,19 +18337,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D300" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D300" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E300" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F300" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -19009,19 +19009,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D321" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D321" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E321" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F321" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -19521,19 +19521,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D337" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D337" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E337" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F337" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -19905,19 +19905,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D349" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D349" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E349" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F349" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -20385,19 +20385,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D364" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D364" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E364" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F364" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -20673,19 +20673,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D373" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D373" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E373" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F373" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -22273,19 +22273,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D423" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D423" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E423" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F423" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -22657,19 +22657,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D435" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D435" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E435" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F435" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -23873,19 +23873,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D473" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D473" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E473" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F473" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -24353,19 +24353,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D488" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D488" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E488" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F488" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -24737,19 +24737,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D500" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D500" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E500" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F500" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -25249,19 +25249,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D516" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D516" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E516" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F516" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -25441,19 +25441,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D522" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D522" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E522" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F522" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -26209,19 +26209,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D546" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D546" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E546" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F546" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -27233,19 +27233,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D578" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D578" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E578" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F578" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -27809,19 +27809,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D596" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D596" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E596" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F596" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -28257,19 +28257,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D610" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D610" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E610" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F610" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -28513,19 +28513,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D618" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D618" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E618" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F618" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -28833,19 +28833,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D628" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D628" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E628" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F628" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -29153,19 +29153,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D638" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D638" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E638" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F638" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -29473,19 +29473,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D648" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D648" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E648" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F648" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -30209,19 +30209,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D671" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D671" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E671" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F671" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -31361,19 +31361,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D707" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D707" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E707" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F707" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -31905,19 +31905,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D724" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D724" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E724" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F724" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -32449,19 +32449,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D741" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D741" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E741" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F741" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -32897,19 +32897,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D755" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D755" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E755" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F755" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -33601,19 +33601,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D777" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D777" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E777" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F777" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -34145,19 +34145,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D794" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D794" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E794" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F794" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -35137,19 +35137,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D825" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D825" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E825" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F825" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -35681,19 +35681,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D842" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D842" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E842" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F842" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -37537,19 +37537,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D900" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D900" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E900" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F900" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -38017,19 +38017,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D915" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D915" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E915" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F915" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -39681,19 +39681,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D967" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D967" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E967" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F967" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -40353,19 +40353,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D988" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D988" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E988" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F988" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -40865,19 +40865,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D1004" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D1004" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E1004" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F1004" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -41185,19 +41185,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D1014" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D1014" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E1014" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F1014" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -41857,19 +41857,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D1035" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D1035" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E1035" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F1035" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -42401,19 +42401,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D1052" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D1052" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E1052" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F1052" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>
@@ -42849,19 +42849,19 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D1066" s="16" t="inlineStr">
-        <is>
-          <t>미노출(검토대상)</t>
+      <c r="D1066" s="17" t="inlineStr">
+        <is>
+          <t>제외(적재제어메타)</t>
         </is>
       </c>
       <c r="E1066" s="11" t="inlineStr">
         <is>
-          <t>낮음(이름기반·P13)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F1066" s="11" t="inlineStr">
         <is>
-          <t>개명·VARIANT param 승격 가능성 — 확정 아님</t>
+          <t>BRONZE 적재 제어 컬럼 — SILVER 미승격 확정(O175)</t>
         </is>
       </c>
     </row>

</xml_diff>